<commit_message>
Latest report and workflows. Version 1.0.0
</commit_message>
<xml_diff>
--- a/CancerSummary/SummaryReports.xlsx
+++ b/CancerSummary/SummaryReports.xlsx
@@ -511,37 +511,37 @@
         <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>35780</v>
+        <v>35701</v>
       </c>
       <c r="D2" t="n">
         <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>10704</v>
+        <v>10672</v>
       </c>
       <c r="F2" t="n">
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>5515</v>
+        <v>5503</v>
       </c>
       <c r="H2" t="n">
         <v>100</v>
       </c>
       <c r="I2" t="n">
-        <v>6826</v>
+        <v>6810</v>
       </c>
       <c r="J2" t="n">
         <v>100</v>
       </c>
       <c r="K2" t="n">
-        <v>7594</v>
+        <v>7581</v>
       </c>
       <c r="L2" t="n">
         <v>100</v>
       </c>
       <c r="M2" t="n">
-        <v>5141</v>
+        <v>5135</v>
       </c>
     </row>
     <row r="3">
@@ -551,37 +551,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>94.73</v>
+        <v>94.94</v>
       </c>
       <c r="C3" t="n">
         <v>33893</v>
       </c>
       <c r="D3" t="n">
-        <v>94.42</v>
+        <v>94.70999999999999</v>
       </c>
       <c r="E3" t="n">
         <v>10107</v>
       </c>
       <c r="F3" t="n">
-        <v>95.45</v>
+        <v>95.66</v>
       </c>
       <c r="G3" t="n">
         <v>5264</v>
       </c>
       <c r="H3" t="n">
-        <v>95.75</v>
+        <v>95.98</v>
       </c>
       <c r="I3" t="n">
         <v>6536</v>
       </c>
       <c r="J3" t="n">
-        <v>94.39</v>
+        <v>94.55</v>
       </c>
       <c r="K3" t="n">
         <v>7168</v>
       </c>
       <c r="L3" t="n">
-        <v>93.72</v>
+        <v>93.83</v>
       </c>
       <c r="M3" t="n">
         <v>4818</v>
@@ -597,37 +597,37 @@
         <v>100</v>
       </c>
       <c r="C4" t="n">
-        <v>35780</v>
+        <v>35701</v>
       </c>
       <c r="D4" t="n">
         <v>100</v>
       </c>
       <c r="E4" t="n">
-        <v>10704</v>
+        <v>10672</v>
       </c>
       <c r="F4" t="n">
         <v>100</v>
       </c>
       <c r="G4" t="n">
-        <v>5515</v>
+        <v>5503</v>
       </c>
       <c r="H4" t="n">
         <v>100</v>
       </c>
       <c r="I4" t="n">
-        <v>6826</v>
+        <v>6810</v>
       </c>
       <c r="J4" t="n">
         <v>100</v>
       </c>
       <c r="K4" t="n">
-        <v>7594</v>
+        <v>7581</v>
       </c>
       <c r="L4" t="n">
         <v>100</v>
       </c>
       <c r="M4" t="n">
-        <v>5141</v>
+        <v>5135</v>
       </c>
     </row>
     <row r="5">
@@ -640,37 +640,37 @@
         <v>100</v>
       </c>
       <c r="C5" t="n">
-        <v>35780</v>
+        <v>35701</v>
       </c>
       <c r="D5" t="n">
         <v>100</v>
       </c>
       <c r="E5" t="n">
-        <v>10704</v>
+        <v>10672</v>
       </c>
       <c r="F5" t="n">
         <v>100</v>
       </c>
       <c r="G5" t="n">
-        <v>5515</v>
+        <v>5503</v>
       </c>
       <c r="H5" t="n">
         <v>100</v>
       </c>
       <c r="I5" t="n">
-        <v>6826</v>
+        <v>6810</v>
       </c>
       <c r="J5" t="n">
         <v>100</v>
       </c>
       <c r="K5" t="n">
-        <v>7594</v>
+        <v>7581</v>
       </c>
       <c r="L5" t="n">
         <v>100</v>
       </c>
       <c r="M5" t="n">
-        <v>5141</v>
+        <v>5135</v>
       </c>
     </row>
     <row r="6">
@@ -683,37 +683,37 @@
         <v>100</v>
       </c>
       <c r="C6" t="n">
-        <v>35780</v>
+        <v>35701</v>
       </c>
       <c r="D6" t="n">
         <v>100</v>
       </c>
       <c r="E6" t="n">
-        <v>10704</v>
+        <v>10672</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
       </c>
       <c r="G6" t="n">
-        <v>5515</v>
+        <v>5503</v>
       </c>
       <c r="H6" t="n">
         <v>100</v>
       </c>
       <c r="I6" t="n">
-        <v>6826</v>
+        <v>6810</v>
       </c>
       <c r="J6" t="n">
         <v>100</v>
       </c>
       <c r="K6" t="n">
-        <v>7594</v>
+        <v>7581</v>
       </c>
       <c r="L6" t="n">
         <v>100</v>
       </c>
       <c r="M6" t="n">
-        <v>5141</v>
+        <v>5135</v>
       </c>
     </row>
     <row r="7">
@@ -726,37 +726,37 @@
         <v>99.15000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>35477</v>
+        <v>35398</v>
       </c>
       <c r="D7" t="n">
         <v>98.72</v>
       </c>
       <c r="E7" t="n">
-        <v>10567</v>
+        <v>10535</v>
       </c>
       <c r="F7" t="n">
         <v>99.02</v>
       </c>
       <c r="G7" t="n">
-        <v>5461</v>
+        <v>5449</v>
       </c>
       <c r="H7" t="n">
         <v>99.27</v>
       </c>
       <c r="I7" t="n">
-        <v>6776</v>
+        <v>6760</v>
       </c>
       <c r="J7" t="n">
         <v>99.5</v>
       </c>
       <c r="K7" t="n">
-        <v>7556</v>
+        <v>7543</v>
       </c>
       <c r="L7" t="n">
         <v>99.53</v>
       </c>
       <c r="M7" t="n">
-        <v>5117</v>
+        <v>5111</v>
       </c>
     </row>
     <row r="8">
@@ -769,37 +769,37 @@
         <v>100</v>
       </c>
       <c r="C8" t="n">
-        <v>35780</v>
+        <v>35701</v>
       </c>
       <c r="D8" t="n">
         <v>100</v>
       </c>
       <c r="E8" t="n">
-        <v>10704</v>
+        <v>10672</v>
       </c>
       <c r="F8" t="n">
         <v>100</v>
       </c>
       <c r="G8" t="n">
-        <v>5515</v>
+        <v>5503</v>
       </c>
       <c r="H8" t="n">
         <v>100</v>
       </c>
       <c r="I8" t="n">
-        <v>6826</v>
+        <v>6810</v>
       </c>
       <c r="J8" t="n">
         <v>100</v>
       </c>
       <c r="K8" t="n">
-        <v>7594</v>
+        <v>7581</v>
       </c>
       <c r="L8" t="n">
         <v>100</v>
       </c>
       <c r="M8" t="n">
-        <v>5141</v>
+        <v>5135</v>
       </c>
     </row>
     <row r="9">
@@ -809,37 +809,37 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>82.20999999999999</v>
+        <v>82.39</v>
       </c>
       <c r="C9" t="n">
         <v>29414</v>
       </c>
       <c r="D9" t="n">
-        <v>64.78</v>
+        <v>64.97</v>
       </c>
       <c r="E9" t="n">
         <v>6934</v>
       </c>
       <c r="F9" t="n">
-        <v>88</v>
+        <v>88.19</v>
       </c>
       <c r="G9" t="n">
         <v>4853</v>
       </c>
       <c r="H9" t="n">
-        <v>89.53</v>
+        <v>89.73999999999999</v>
       </c>
       <c r="I9" t="n">
         <v>6111</v>
       </c>
       <c r="J9" t="n">
-        <v>92.51000000000001</v>
+        <v>92.67</v>
       </c>
       <c r="K9" t="n">
         <v>7025</v>
       </c>
       <c r="L9" t="n">
-        <v>87.36</v>
+        <v>87.45999999999999</v>
       </c>
       <c r="M9" t="n">
         <v>4491</v>
@@ -852,37 +852,37 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>29.53</v>
+        <v>29.6</v>
       </c>
       <c r="C10" t="n">
         <v>10566</v>
       </c>
       <c r="D10" t="n">
-        <v>28.24</v>
+        <v>28.33</v>
       </c>
       <c r="E10" t="n">
         <v>3023</v>
       </c>
       <c r="F10" t="n">
-        <v>37.04</v>
+        <v>37.13</v>
       </c>
       <c r="G10" t="n">
         <v>2043</v>
       </c>
       <c r="H10" t="n">
-        <v>33.53</v>
+        <v>33.61</v>
       </c>
       <c r="I10" t="n">
         <v>2289</v>
       </c>
       <c r="J10" t="n">
-        <v>27.68</v>
+        <v>27.73</v>
       </c>
       <c r="K10" t="n">
         <v>2102</v>
       </c>
       <c r="L10" t="n">
-        <v>21.57</v>
+        <v>21.6</v>
       </c>
       <c r="M10" t="n">
         <v>1109</v>
@@ -895,37 +895,37 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>48.87</v>
+        <v>48.98</v>
       </c>
       <c r="C11" t="n">
         <v>17485</v>
       </c>
       <c r="D11" t="n">
-        <v>47.69</v>
+        <v>47.84</v>
       </c>
       <c r="E11" t="n">
         <v>5105</v>
       </c>
       <c r="F11" t="n">
-        <v>47.91</v>
+        <v>48.01</v>
       </c>
       <c r="G11" t="n">
         <v>2642</v>
       </c>
       <c r="H11" t="n">
-        <v>52.2</v>
+        <v>52.32</v>
       </c>
       <c r="I11" t="n">
         <v>3563</v>
       </c>
       <c r="J11" t="n">
-        <v>53.48</v>
+        <v>53.57</v>
       </c>
       <c r="K11" t="n">
         <v>4061</v>
       </c>
       <c r="L11" t="n">
-        <v>41.12</v>
+        <v>41.17</v>
       </c>
       <c r="M11" t="n">
         <v>2114</v>
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1119</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="9">
@@ -2441,7 +2441,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1616</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="10">
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11">
@@ -2491,7 +2491,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>303</v>
+        <v>287</v>
       </c>
     </row>
     <row r="15">
@@ -2541,7 +2541,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="20">
@@ -2691,7 +2691,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="35">
@@ -2721,7 +2721,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38">
@@ -2751,7 +2751,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>340</v>
+        <v>316</v>
       </c>
     </row>
     <row r="41">
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>620</v>
+        <v>615</v>
       </c>
     </row>
     <row r="42">
@@ -2781,7 +2781,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44">
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3815</v>
+        <v>3736</v>
       </c>
     </row>
     <row r="9">
@@ -3607,4 +3607,246 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019242F544423A8439CBDDB55F90E1A09" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="735290c03c6af11b8253c59e024f788a">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9d9492b0-01d7-479c-9e6d-86db3c4557e3" xmlns:ns3="2cd82415-e45a-43fa-87d5-b2ae2acda126" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e151c7a5b126992fa047db59ef20defe" ns2:_="" ns3:_="">
+    <xsd:import namespace="9d9492b0-01d7-479c-9e6d-86db3c4557e3"/>
+    <xsd:import namespace="2cd82415-e45a-43fa-87d5-b2ae2acda126"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9d9492b0-01d7-479c-9e6d-86db3c4557e3" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="10" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="12" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="ad4fd8df-27a2-471a-8ee0-838121336595" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="13" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="16" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="19" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2cd82415-e45a-43fa-87d5-b2ae2acda126" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="17" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="18" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d9492b0-01d7-479c-9e6d-86db3c4557e3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60A173B5-000F-45E3-8D87-76C15906A705}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B99D762-ED4A-4BFD-B280-09471E823A2B}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBFACBD3-1030-41FF-BA74-24B489E5CF35}"/>
 </file>
</xml_diff>